<commit_message>
security: untrack output directory, update exam grading rules and UI enhancements
</commit_message>
<xml_diff>
--- a/slides/uet-oop-midterm-2025-2026-INT2204-80.xlsx
+++ b/slides/uet-oop-midterm-2025-2026-INT2204-80.xlsx
@@ -848,7 +848,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>C1.1</t>
@@ -872,17 +871,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
           <t>Sai</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" t="inlineStr">
@@ -895,7 +888,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>C1.2</t>
@@ -919,17 +911,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" t="inlineStr">
@@ -942,7 +928,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>C1.3</t>
@@ -966,17 +951,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" t="inlineStr">
@@ -989,7 +968,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>C1.4</t>
@@ -1013,17 +991,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" t="inlineStr">
@@ -1036,7 +1008,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>C1.5</t>
@@ -1060,17 +1031,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr">
         <is>
           <t>Sai</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -1083,7 +1048,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>C1.6</t>
@@ -1107,17 +1071,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>Sai</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -1130,7 +1088,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
           <t>C1.7</t>
@@ -1154,17 +1111,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" t="inlineStr">
@@ -1177,7 +1128,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>C1.8</t>
@@ -1201,17 +1151,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
           <t>Sai</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -1224,7 +1168,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>C1.9</t>
@@ -1248,17 +1191,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>Sai</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -1271,7 +1208,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>C1.10</t>
@@ -1295,17 +1231,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -1318,7 +1248,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>C1.11</t>
@@ -1342,17 +1271,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" t="inlineStr">
@@ -1365,7 +1288,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>C1.12</t>
@@ -1389,17 +1311,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" t="inlineStr">
@@ -1412,7 +1328,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
           <t>C1.13</t>
@@ -1436,17 +1351,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" t="inlineStr">
@@ -1459,7 +1368,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
           <t>C1.14</t>
@@ -1483,17 +1391,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
           <t>Sai</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" t="inlineStr">
@@ -1506,7 +1408,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
           <t>C1.15</t>
@@ -1530,17 +1431,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" t="inlineStr">
@@ -1553,7 +1448,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
           <t>C1.16</t>
@@ -1577,17 +1471,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>Sai</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" t="inlineStr">
@@ -1600,7 +1488,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
           <t>C1.17</t>
@@ -1624,17 +1511,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr">
         <is>
           <t>Sai</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" t="inlineStr">
@@ -1647,7 +1528,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>C1.18</t>
@@ -1671,17 +1551,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" t="inlineStr">
@@ -1694,7 +1568,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>C1.19</t>
@@ -1718,17 +1591,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>Sai</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" t="inlineStr">
@@ -1741,7 +1608,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>C1.20</t>
@@ -1765,17 +1631,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" t="inlineStr">
@@ -1788,7 +1648,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>C1.21</t>
@@ -1812,17 +1671,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr">
         <is>
           <t>Sai</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23" ht="60" customHeight="1">
       <c r="A23" t="inlineStr">
@@ -1835,7 +1688,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>C1.22</t>
@@ -1859,17 +1711,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24" ht="60" customHeight="1">
       <c r="A24" t="inlineStr">
@@ -1882,7 +1728,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>C1.23</t>
@@ -1906,17 +1751,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25" ht="60" customHeight="1">
       <c r="A25" t="inlineStr">
@@ -1929,7 +1768,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>C1.24</t>
@@ -1953,17 +1791,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26" ht="60" customHeight="1">
       <c r="A26" t="inlineStr">
@@ -1976,7 +1808,6 @@
           <t>Câu 1 - Đúng/Sai (5 điểm)</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>C1.25</t>
@@ -2000,17 +1831,11 @@
           <t>auto</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>Đúng</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27" ht="60" customHeight="1">
       <c r="A27" t="inlineStr">
@@ -2023,7 +1848,6 @@
           <t>Câu 2 - Tự luận (1,5 điểm)</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>C2.a</t>
@@ -2047,11 +1871,6 @@
           <t>llm_assisted</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
           <t>Overriding xảy ra giữa lớp cha - con (cùng tên, cùng tham số, cùng kiểu trả về, quyết định lúc runtime - dynamic binding). Overloading xảy ra trong cùng lớp hoặc lớp con (cùng tên, khác danh sách tham số, quyết định lúc compile-time - static binding). Cần có mã Java minh họa hợp lệ cho cả hai.</t>
@@ -2074,7 +1893,6 @@
           <t>Câu 2 - Tự luận (1,5 điểm)</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>C2.b</t>
@@ -2098,11 +1916,6 @@
           <t>llm_assisted</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
           <t>Khác biệt: Abstract class hỗ trợ đơn kế thừa, chứa thuộc tính biến, constructor, phương thức có/không có thân hàm. Interface hỗ trợ đa kế thừa (implements nhiều interface), thuộc tính mặc định public static final, không constructor, chứa phương thức abstract/default/static. Ngữ cảnh: Dùng Abstract Class khi các lớp có quan hệ họ hàng close is-a và chia sẻ mã/trạng thái chung. Dùng Interface khi định nghĩa hợp đồng hành vi (can-do) cho các lớp không nhất thiết có quan hệ kế thừa.</t>
@@ -2125,7 +1938,6 @@
           <t>Câu 3 - Một lựa chọn (2 điểm)</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>C3.1</t>
@@ -2178,8 +1990,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30" ht="60" customHeight="1">
       <c r="A30" t="inlineStr">
@@ -2192,7 +2002,6 @@
           <t>Câu 3 - Một lựa chọn (2 điểm)</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>C3.2</t>
@@ -2241,8 +2050,6 @@
           <t>C</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31" ht="60" customHeight="1">
       <c r="A31" t="inlineStr">
@@ -2255,7 +2062,6 @@
           <t>Câu 3 - Một lựa chọn (2 điểm)</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>C3.3</t>
@@ -2304,8 +2110,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32" ht="60" customHeight="1">
       <c r="A32" t="inlineStr">
@@ -2318,7 +2122,6 @@
           <t>Câu 3 - Một lựa chọn (2 điểm)</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>C3.4</t>
@@ -2367,8 +2170,6 @@
           <t>B</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33" ht="60" customHeight="1">
       <c r="A33" t="inlineStr">
@@ -2381,7 +2182,6 @@
           <t>Câu 3 - Một lựa chọn (2 điểm)</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>C3.5</t>
@@ -2430,8 +2230,6 @@
           <t>C</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34" ht="220" customHeight="1">
       <c r="A34" t="inlineStr">
@@ -2500,7 +2298,8 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Chương trình Java trên có những lỗi biên dịch nào? Hãy chỉ ra các câu lệnh gây lỗi, giải thích nguyên nhân và đưa ra phương án sửa để chương trình biên dịch thành công.</t>
+          <t>Chương trình Java trên có chứa các lỗi biên dịch. Hãy chỉ ra các câu lệnh gây lỗi, giải thích nguyên nhân và đưa ra phương án sửa để chương trình biên dịch thành công.
+(Quy định chấm: Thí sinh chỉ cần chỉ ra VÀ SỬA ĐÚNG ít nhất 3 lỗi sai sẽ đạt điểm tối đa 1.0 điểm. Nếu chỉ phát hiện đúng lỗi mà không đưa ra phương án sửa hợp lệ thì chỉ nhận 50% số điểm của lỗi đó - 0.167 điểm/lỗi).</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -2511,24 +2310,27 @@
           <t>llm_assisted</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Các lỗi biên dịch:
+          <t>Danh sách 5 lỗi biên dịch:
 1. Rectangle(double, double) ngầm gọi super() nhưng Shape không có constructor không tham số.
-2. Trong Rectangle(String, double, double), super(c) phải là câu lệnh đầu tiên trong constructor.
-3. Từ khóa Public viết hoa P trong getArea() là sai cú pháp (phải là public).
+2. In Rectangle(String, double, double), super(c) phải là câu lệnh đầu tiên trong constructor.
+3. Từ khóa Public viết hoa P trong getArea() là sai cú pháp (phải viết thường public).
 4. Lớp Circle kế thừa Shape nhưng không override phương thức trừu tượng getArea().
-5. Trong main: Shape s1 = new Shape("Red"); vi phạm không được khởi tạo trực tiếp đối tượng từ abstract class.</t>
+5. In main: Shape s1 = new Shape("Red"); vi phạm không được khởi tạo trực tiếp đối tượng từ abstract class.
+Quy định chấm điểm cho Câu 4.a (tổng điểm tối đa 1.0):
+- Sinh viên tìm và sửa đúng 1 lỗi: 0.333 điểm (nếu chỉ tìm đúng lỗi mà không sửa / sửa sai: 0.167 điểm).
+- Sinh viên tìm và sửa đúng 2 lỗi: 0.667 điểm (nếu chỉ tìm đúng lỗi mà không sửa / sửa sai: 0.333 điểm).
+- Sinh viên tìm và sửa đúng từ 3 lỗi trở lên: 1.0 điểm (đạt điểm tối đa).
+- Mỗi lỗi nếu chỉ chỉ ra đúng mà không đưa ra phương án sửa hợp lệ: chỉ tính 50% số điểm của lỗi đó.</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Đối chiếu tính chính xác khi chỉ ra lỗi biên dịch, giải thích nguyên nhân và phương án sửa hợp lệ.</t>
+          <t>Chấm bài tự động/LLM cho câu 4.a theo quy định:
+1. Đoạn mã chứa 5 lỗi biên dịch tiềm năng.
+2. Mỗi lỗi sinh viên chỉ ra VÀ SỬA ĐÚNG được cộng 0.333 điểm. Nếu sinh viên chỉ phát hiện đúng dòng lỗi/nguyên nhân mà KHÔNG SỬA được hoặc SỬA SAI thì chỉ tính 50% điểm của lỗi đó (0.167 điểm/lỗi).
+3. Tổng điểm C4.a = Min(1.0, Tổng điểm các lỗi đạt được). Sinh viên chỉ cần chỉ ra VÀ SỬA ĐÚNG từ 3 lỗi trở lên sẽ nhận điểm tối đa 1.0 điểm.</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2345,6 @@
           <t>Câu 4 - Đọc và sửa mã Java (1,5 điểm)</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>C4.b</t>
@@ -2567,11 +2368,6 @@
           <t>llm_assisted</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
           <t>Kết quả in ra màn hình: Color: Blue, Area: 20.0
@@ -2618,7 +2414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2732,17 +2528,17 @@
     <row r="6" ht="42" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C4.a</t>
+          <t>C4.b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>constructor-super</t>
+          <t>correct-output</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Phát hiện lỗi thiếu super() mặc định trong Rectangle(w,h) và super(c) không đứng ở vị trí đầu tiên</t>
+          <t>Xác định đúng chuỗi kết quả in ra màn hình: Color: Blue, Area: 20.0</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -2752,17 +2548,17 @@
     <row r="7" ht="42" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C4.a</t>
+          <t>C4.b</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>syntax-keyword</t>
+          <t>dynamic-binding</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Phát hiện lỗi cú pháp từ khóa Public viết hoa ở phương thức getArea() trong Rectangle</t>
+          <t>Giải thích đúng cơ chế liên kết động (dynamic binding / polymorphism) khi gọi getArea()</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -2777,16 +2573,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>abstract-method</t>
+          <t>error-1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Phát hiện lỗi lớp Circle kế thừa Shape nhưng chưa override phương thức trừu tượng getArea()</t>
+          <t>Chỉ ra và sửa đúng lỗi biên dịch thứ 1 (0.333đ; chỉ chỉ ra không sửa: 0.167đ)</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.25</v>
+        <v>0.333</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
@@ -2797,58 +2593,39 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>abstract-instantiation</t>
+          <t>error-2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Phát hiện lỗi khởi tạo đối tượng trực tiếp từ abstract class Shape trong hàm main</t>
+          <t>Chỉ ra và sửa đúng lỗi biên dịch thứ 2 (0.333đ; chỉ chỉ ra không sửa: 0.167đ)</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.25</v>
+        <v>0.333</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C4.b</t>
+          <t>C4.a</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>correct-output</t>
+          <t>error-3</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Xác định đúng chuỗi kết quả in ra màn hình: Color: Blue, Area: 20.0</t>
+          <t>Chỉ ra và sửa đúng lỗi biên dịch thứ 3 (đạt điểm tối đa 1.0 điểm khi tìm &amp; sửa đúng &gt;= 3 lỗi)</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>C4.b</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>dynamic-binding</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Giải thích đúng cơ chế liên kết động (dynamic binding / polymorphism) khi gọi getArea()</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
+        <v>0.334</v>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1"/>
     <row r="12" ht="42" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:D12"/>

</xml_diff>